<commit_message>
[24차] 간단히 Tutorial1Group 3차 편집
이번엔 두 스크립트만 수정했습니다.

JangYoungSim은 E 상호작용 후 Surprised를 마지막 프레임으로 강제 샘플링하고 Animator.speed = 0으로 멈춥니다. 이동 잠금이 다시 걸려도 one-shot 상태면 Idle을 재생하지 않게 막았습니다.

CommonSkipButton_Tutorial1은 런타임에 Tutorial1Group > Tutorial1Background 아래로 생성되며, 월드 스페이스 버튼으로 전환됩니다. 카메라 기준 오른쪽 상단을 따라가되 Tutorial1Background의 bounds 밖으로는 나가지 않도록 매 프레임 클램프합니다.
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/OO_Tutorial.xlsx
+++ b/JsonConverter/ExcelFiles/OO_Tutorial.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
   <si>
     <t>캐릭터 고유 ID</t>
   </si>
@@ -70,10 +70,6 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>narration_tutorial_03</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
     <t>튜토리얼 가이드1</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
@@ -91,6 +87,18 @@
   </si>
   <si>
     <t>WASD를 눌러 캐릭터를 움직여보세요! 앉아 있는 목각인형을 찾아 E를 누르시고 임무를 완수하세요.</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>튜토리얼 가이드2</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>배고픈 재익이 음식을 찾고 있습니다. Space바를 눌러 점프할 수 있습니다! 음식과 상호작용 키는 E입니다.</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>narration_tutorial_03</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -567,10 +575,10 @@
         <v>13</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
@@ -587,13 +595,13 @@
     </row>
     <row r="5" spans="1:15" ht="15.75" customHeight="1">
       <c r="A5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="C5" s="6" t="s">
         <v>17</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>18</v>
       </c>
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
@@ -610,10 +618,14 @@
     </row>
     <row r="6" spans="1:15" ht="15.75" customHeight="1">
       <c r="A6" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
+        <v>21</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>20</v>
+      </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>

</xml_diff>